<commit_message>
updated function definitions file.
</commit_message>
<xml_diff>
--- a/docs/tracker功能定义.xlsx
+++ b/docs/tracker功能定义.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\works\solutions\GPS-Tracker\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\works\solutions\GPS-Tracker\source-code\tracker\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BC0B8E0-DA70-4738-95C9-B0A3DB56E32D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4366522E-2716-40B1-B77B-98934258B64E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F8AC9A2B-7803-4AB1-93AC-DD66ED057729}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="65">
   <si>
     <t>功能</t>
   </si>
@@ -171,10 +171,6 @@
       <t>发送短信。
 报警代码：50001</t>
     </r>
-  </si>
-  <si>
-    <t>网络畅通时，需第一时间将报警信息报给云端，同时发送报警短信到内置的电话号码。
-在网络不通时，需将事件发生时间和故障代码存入文件系统，待网络恢复时，报给云端，并短信通知内置的电话号码。</t>
   </si>
   <si>
     <t>远程配置或控制</t>
@@ -702,75 +698,6 @@
   </si>
   <si>
     <r>
-      <t>上电时，待网络连接后，检测是否需要更新升级。
-是的话：若非自动升级，则下载升级包，并将升级包准备完毕的通知报给云端；在云端或手机APP上控制设备执行升级操作；升级完毕后，将升级状态报告给云端。
-功能的开启，可由云端或手机APP控制。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>默认开启</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>该功能。
-功能开启的状态下，可由</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="8" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>云端或手机APP</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>配置是否自动升级。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>默认自动升级</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>。</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>设备在开机自检或正常工作中遇到了故障时报警。
 功能的开启，可由</t>
     </r>
@@ -1195,12 +1122,102 @@
       <t>远程控制固件升级的流程。</t>
     </r>
   </si>
+  <si>
+    <t>云端功能</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">网络畅通时，需第一时间将报警信息报给云端，同时发送报警短信到内置的电话号码。
+在网络不通时，需将事件发生时间和故障代码存入文件系统，待网络恢复时，报给云端，并短信通知内置的电话号码。
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（考虑删除振动报警）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>上电时，待网络连接后，检测是否需要更新升级。
+是的话：若非自动升级，则上云端上报有新的更新；在云端或手机APP点击下载按钮；下载升级包，并将升级包准备完毕的通知报给云端；在云端或手机APP上控制设备执行升级操作；升级完毕后，将升级状态报告给云端。
+功能的开启，可由云端或手机APP控制。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>默认开启</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>该功能。
+功能开启的状态下，可由</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="8" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>云端或手机APP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>配置是否自动升级。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>默认自动升级</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>。</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1288,6 +1305,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1309,7 +1334,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1326,6 +1351,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1678,7 +1704,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C3" s="1"/>
     </row>
@@ -1696,7 +1722,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" s="1"/>
     </row>
@@ -1705,7 +1731,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>12</v>
@@ -1725,7 +1751,7 @@
         <v>13</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="75" x14ac:dyDescent="0.25">
@@ -1733,10 +1759,10 @@
         <v>14</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -1744,7 +1770,10 @@
         <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -1752,7 +1781,7 @@
         <v>16</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C11" t="s">
         <v>20</v>
@@ -1763,7 +1792,7 @@
         <v>17</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C12" t="s">
         <v>20</v>
@@ -1788,12 +1817,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -1801,10 +1830,10 @@
         <v>24</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>33</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="60" x14ac:dyDescent="0.25">
@@ -1812,7 +1841,7 @@
         <v>25</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C17" s="5"/>
     </row>
@@ -1821,7 +1850,7 @@
         <v>26</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C18" s="5"/>
     </row>
@@ -1830,7 +1859,7 @@
         <v>27</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C19" s="5"/>
     </row>
@@ -1839,7 +1868,7 @@
         <v>28</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C20" s="5"/>
     </row>
@@ -1848,7 +1877,7 @@
         <v>29</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C21" s="5"/>
     </row>
@@ -1857,7 +1886,7 @@
         <v>30</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C22" s="5"/>
     </row>
@@ -1874,10 +1903,10 @@
     </row>
     <row r="24" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C24" t="s">
         <v>20</v>
@@ -1903,18 +1932,18 @@
   <sheetData>
     <row r="1" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="405" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1933,26 +1962,26 @@
   <sheetData>
     <row r="1" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
1. updated function definitions file 2. add tracker-specification.xlsx
</commit_message>
<xml_diff>
--- a/docs/tracker功能定义.xlsx
+++ b/docs/tracker功能定义.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\works\solutions\GPS-Tracker\source-code\tracker\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4366522E-2716-40B1-B77B-98934258B64E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD0E498D-2E1B-46F9-A9A4-C875B78FC9E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F8AC9A2B-7803-4AB1-93AC-DD66ED057729}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{F8AC9A2B-7803-4AB1-93AC-DD66ED057729}"/>
   </bookViews>
   <sheets>
     <sheet name="功能描述" sheetId="1" r:id="rId1"/>
@@ -939,54 +939,6 @@
   </si>
   <si>
     <r>
-      <t>检测到较强振动时报警。
-功能的开启，可由</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="8" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>云端或手机APP控制</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>默认关闭</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>该功能。
-报警代码：30006</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>检测到急起急停或急转弯时，报驾驶行为异常。
 功能的开启，可由</t>
     </r>
@@ -1146,8 +1098,29 @@
   <si>
     <r>
       <t>上电时，待网络连接后，检测是否需要更新升级。
-是的话：若非自动升级，则上云端上报有新的更新；在云端或手机APP点击下载按钮；下载升级包，并将升级包准备完毕的通知报给云端；在云端或手机APP上控制设备执行升级操作；升级完毕后，将升级状态报告给云端。
-功能的开启，可由云端或手机APP控制。</t>
+是的话：若非自动升级，则上云端上报有新的更新；在云端或手机APP点击升级按钮，设备开启进行升级；升级完毕后，将升级状态报告给云端。
+功能的开启，可由</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>云端或手机APP控制</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>。</t>
     </r>
     <r>
       <rPr>
@@ -1210,6 +1183,58 @@
         <scheme val="minor"/>
       </rPr>
       <t>。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>检测到较强振动时报警。
+功能的开启，可由</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <strike/>
+        <sz val="11"/>
+        <color theme="8" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>云端或手机APP控制</t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>。</t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>默认关闭</t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>该功能。
+报警代码：30006</t>
     </r>
   </si>
 </sst>
@@ -1217,7 +1242,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1313,6 +1338,39 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <strike/>
+      <sz val="11"/>
+      <color theme="8" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1334,7 +1392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1345,13 +1403,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1772,8 +1833,8 @@
       <c r="B10" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>62</v>
+      <c r="C10" s="4" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -1817,12 +1878,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -1832,8 +1893,8 @@
       <c r="B16" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>63</v>
+      <c r="C16" s="5" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="60" x14ac:dyDescent="0.25">
@@ -1843,7 +1904,7 @@
       <c r="B17" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C17" s="5"/>
+      <c r="C17" s="6"/>
     </row>
     <row r="18" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
@@ -1852,7 +1913,7 @@
       <c r="B18" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C18" s="5"/>
+      <c r="C18" s="6"/>
     </row>
     <row r="19" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
@@ -1861,7 +1922,7 @@
       <c r="B19" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C19" s="5"/>
+      <c r="C19" s="6"/>
     </row>
     <row r="20" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
@@ -1870,25 +1931,25 @@
       <c r="B20" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C20" s="5"/>
+      <c r="C20" s="6"/>
     </row>
     <row r="21" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C21" s="5"/>
+      <c r="B21" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C21" s="6"/>
     </row>
     <row r="22" spans="1:3" ht="105" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C22" s="5"/>
+        <v>59</v>
+      </c>
+      <c r="C22" s="6"/>
     </row>
     <row r="23" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
@@ -1906,7 +1967,7 @@
         <v>33</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C24" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
updated settings.py & function definitions file
</commit_message>
<xml_diff>
--- a/docs/tracker功能定义.xlsx
+++ b/docs/tracker功能定义.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\works\solutions\GPS-Tracker\source-code\tracker\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39628506-76FF-431A-8B30-D5EFFF6AA013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{276F1630-47C5-4311-8D1A-9A0A99E8447D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{F8AC9A2B-7803-4AB1-93AC-DD66ED057729}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F8AC9A2B-7803-4AB1-93AC-DD66ED057729}"/>
   </bookViews>
   <sheets>
     <sheet name="功能描述" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="61">
   <si>
     <t>功能</t>
   </si>
@@ -83,9 +83,6 @@
   </si>
   <si>
     <t>多重定位</t>
-  </si>
-  <si>
-    <t>电子围栏</t>
   </si>
   <si>
     <t>语音监听</t>
@@ -135,9 +132,6 @@
   </si>
   <si>
     <t>拆卸报警</t>
-  </si>
-  <si>
-    <t>振动报警</t>
   </si>
   <si>
     <t>SOS一键报警</t>
@@ -552,54 +546,6 @@
   </si>
   <si>
     <r>
-      <t>由云端规划安全区域或航线。
-位置超出区域或偏离航线的，云端向登记的手机号发送报警短信。
-功能的开启，可由</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="8" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>云端或手机APP控制</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>默认开启</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>该功能。</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>云端登记的手机号拨打tracker中的手机号时，自动接听，监听现场的声音。
 功能的开启，可由</t>
     </r>
@@ -891,112 +837,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="8" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>远程配置</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>：电话号码、远程配置定位器工作模式、定位使用的技术手段、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>语音监听、自动录音上报、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">固件升级及自动升级、故障报警、低电报警、超速报警、拔卡报警、拆卸报警、振动报警和驾驶行为监测功能的开关。
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="8" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>远程控制</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>远程控制录音并上报、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>远程控制固件升级的流程。</t>
-    </r>
-  </si>
-  <si>
-    <t>云端功能</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">网络畅通时，需第一时间将报警信息报给云端，同时发送报警短信到内置的电话号码。
-在网络不通时，需将事件发生时间和故障代码存入文件系统，待网络恢复时，报给云端，并短信通知内置的电话号码。
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>（考虑删除振动报警）</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>上电时，待网络连接后，检测是否需要更新升级。
 是的话：若非自动升级，则上云端上报有新的更新；在云端或手机APP点击升级按钮，设备开启进行升级；升级完毕后，将升级状态报告给云端。
 功能的开启，可由</t>
@@ -1087,58 +927,6 @@
   </si>
   <si>
     <r>
-      <t>检测到较强振动时报警。
-功能的开启，可由</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <strike/>
-        <sz val="11"/>
-        <color theme="8" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>云端或手机APP控制</t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>。</t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>默认关闭</t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>该功能。
-报警代码：30006</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>电量低于设定值时报警。
 低电的阈值默认为5%，可由</t>
     </r>
@@ -1252,13 +1040,102 @@
       <t>该功能。
 报警代码：30003</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="8" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>远程配置</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>：电话号码、定位使用的技术手段、远程配置定位器工作模式、定位的周期、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>语音监听、自动录音上报、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">固件升级及自动升级、故障报警、低电报警、超速报警、拔卡报警、拆卸报警、振动报警和驾驶行为监测功能的开关。
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="8" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>远程控制</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>远程控制录音并上报、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>远程控制固件升级的流程。</t>
+    </r>
+  </si>
+  <si>
+    <t>网络畅通时，需第一时间将报警信息报给云端，同时发送报警短信到内置的电话号码。
+在网络不通时，需将事件发生时间和故障代码存入文件系统，待网络恢复时，报给云端，并短信通知内置的电话号码。</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1349,47 +1226,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FF0070C0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <strike/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <strike/>
-      <sz val="11"/>
-      <color theme="8" tint="-0.249977111117893"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <strike/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1415,7 +1252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1426,8 +1263,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1435,9 +1271,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1758,7 +1591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A79593AC-26FC-4BA1-97DA-24B839142EBD}">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
@@ -1791,7 +1624,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C3" s="1"/>
     </row>
@@ -1803,7 +1636,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1811,7 +1644,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C5" s="1"/>
     </row>
@@ -1820,7 +1653,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>12</v>
@@ -1840,7 +1673,7 @@
         <v>13</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="75" x14ac:dyDescent="0.25">
@@ -1848,162 +1681,142 @@
         <v>14</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="105" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="6"/>
+    </row>
+    <row r="17" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" s="6"/>
+    </row>
+    <row r="18" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C12" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="105" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="C17" s="7"/>
-    </row>
-    <row r="18" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="C18" s="7"/>
+      <c r="C18" s="6"/>
     </row>
     <row r="19" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C19" s="7"/>
-    </row>
-    <row r="20" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="C19" s="6"/>
+    </row>
+    <row r="20" spans="1:3" ht="105" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="6"/>
+    </row>
+    <row r="21" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C20" s="7"/>
-    </row>
-    <row r="21" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
+      <c r="B21" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C21" s="7"/>
-    </row>
-    <row r="22" spans="1:3" ht="105" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>64</v>
+        <v>30</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C22" s="7"/>
-    </row>
-    <row r="23" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C24" t="s">
-        <v>20</v>
+        <v>59</v>
+      </c>
+      <c r="C22" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C16:C22"/>
+    <mergeCell ref="C15:C20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2021,18 +1834,18 @@
   <sheetData>
     <row r="1" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="405" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2051,26 +1864,26 @@
   <sheetData>
     <row r="1" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
         <v>45</v>
-      </c>
-      <c r="C1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>